<commit_message>
feat(scraper): robustecer recolección y evitar reprocesamiento de leads existentes
Agrega tolerancia a fichas de Google Maps que no cargan (timeout + skip automático)
Implementa navegación segura de retorno al listado para evitar bloqueos
Simplifica collector: elimina validación externa por websites/wa.me/api.whatsapp.com
Añade normalización local de teléfono en collector y clasificación por teléfono
Incorpora filtro previo de teléfonos existentes en SQLite para omitir negocios ya guardados
Agrega get_existing_phones() en storage y lo integra en main.py
Crea PROJECT.MD como memoria de contexto del proyecto
Añade .gitignore con reglas para Python, Excel, DB y archivos Markdown temporales`
</commit_message>
<xml_diff>
--- a/leads_jercol_rest.xlsx
+++ b/leads_jercol_rest.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -535,14 +535,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LEADS - RESTAURANTES EN MONTERIA COLOMBIA - 26/03/2026</t>
+          <t>LEADS - RESTAURANTES EN MONTERIA COLOMBIA - 27/03/2026</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total encontrados: 3  |  Con WhatsApp confirmado: 1  |  WhatsApp probable: 2  |  Generado por Jercol Technologies</t>
+          <t>Total encontrados: 4  |  Con WhatsApp confirmado: 2  |  WhatsApp probable: 2  |  Generado por Jercol Technologies</t>
         </is>
       </c>
     </row>
@@ -735,6 +735,52 @@
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Los Potrillos Restaurante-Bar</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Restaurante familiar</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>3105974885</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Km 59+700 RN 7401, Montería, Córdoba</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/lospotrillosrestaurantebar</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -751,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -884,6 +930,36 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Los Potrillos Restaurante-Bar</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3105974885</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Km 59+700 RN 7401, Montería, Córdoba</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/lospotrillosrestaurantebar</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>